<commit_message>
Agent test runs, fixes from them, and skill packaging
Four end-to-end runs by fresh Claude agents (draft and role emails,
absences, bargaining sheet, ambiguous and overflowing absences) passed
22 of 22 checks against reference results. Fixes from what the agents
reported: the pairing skill asks on class day whether role emails went
out when roles aren't recorded as sent; absent students are listed under
their own role; the bargaining sheet's main tab is named "Week N
Simulation"; a redundant logging instruction is removed.

Adds shared/package_skills.py, which validates each skill and writes
dist/<skill>.zip for upload to the Claude desktop app (dist/ ignored).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/negotiation_agent/examples/BUS 4489 F26 Roster - Used Car drafted.xlsx
+++ b/negotiation_agent/examples/BUS 4489 F26 Roster - Used Car drafted.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Att - Fall" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Att - Spring" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="E1" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="UC" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="SL" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Att - Fall" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Att - Spring" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="E1" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UC" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SL" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>